<commit_message>
Add Argus cashflow import + top-line income parity
- read_argus_cashflow_xls() parses Argus Enterprise Cash Flow .xls
  exports; verified on 5 deals (xlrd>=2.0 added)
- argus_top_line_income() reporter builds Argus's 16-row block from a
  projection, wired into the workbook as a new top_line_income sheet
- Validation deal validation/argus_unbound.py + tests/test_argus_unbound.py
  pin Y1..Y10 dollar-for-dollar parity vs the Argus Unbound Gateway export
  (every row within $25; Y11 excluded for rollover modeling reasons)
- opex_with_pct_of_revenue_fee() iteratively solves Argus's %-of-EGR
  property management fee — closes the input-construction gap that
  caused an apparent 12% Y1 recovery drift on Unbound
- PBR convention fix: zero renewal_market_discount_pct in the perfect
  rent-roll re-projection so PBR uses the at-market new-tenant rate

133 -> 205 tests.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sample_workbook.xlsx
+++ b/docs/sample_workbook.xlsx
@@ -26,12 +26,13 @@
     <sheet name="mark_to_market" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="cashflows" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="annual_summary" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="reversion" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="irr_summary" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="yield_matrix" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="sensitivity" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="waterfall_schedule" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="waterfall_summary" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="top_line_income" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="reversion" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="irr_summary" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="yield_matrix" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="sensitivity" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="waterfall_schedule" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="waterfall_summary" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -41,8 +42,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -73,9 +74,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -441,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B36"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,7 +513,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
@@ -687,7 +688,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
@@ -722,102 +722,113 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>reversion</t>
+          <t>top_line_income</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Terminal NOI, gross/net sale, loan payoff, net-to-equity, basis used</t>
+          <t>Argus-style top-line income block (Potential Base Rent → Effective Gross Revenue). Rows mirror the Argus 'Cash Flow' report; columns are fiscal years anchored on acquisition_date.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>irr_summary</t>
+          <t>reversion</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Unlevered + levered IRR under monthly_annualized, annual_end_of_year, annual_mid_year conventions. Plus equity multiples.</t>
+          <t>Terminal NOI, gross/net sale, loan payoff, net-to-equity, basis used</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>sensitivity</t>
+          <t>irr_summary</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>5x5 grid: exit cap rate (rows) × acquisition price (cols), unlevered IRR cells (mid-year convention)</t>
+          <t>Unlevered + levered IRR under monthly_annualized, annual_end_of_year, annual_mid_year conventions. Plus equity multiples.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>sensitivity</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>5x5 grid: exit cap rate (rows) × acquisition price (cols), unlevered IRR cells (mid-year convention)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>yield_matrix</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>Year-by-year going-in / current yield: NOI / acquisition price</t>
-        </is>
-      </c>
-    </row>
-    <row r="31"/>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>ARGUS PARITY</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Reversion</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Set timing!reversion_basis = 'forward' to match Argus's year-N+1 / exit-cap convention. 'trailing' = trailing-12 / exit-cap.</t>
+          <t>ARGUS PARITY</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>IRR</t>
+          <t>Reversion</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Argus reports mid-year IRR by default. See irr_summary.annual_mid_year.</t>
+          <t>Set timing!reversion_basis = 'forward' to match Argus's year-N+1 / exit-cap convention. 'trailing' = trailing-12 / exit-cap.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>MLA blending</t>
+          <t>IRR</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>OpenVal blends renewal / new-tenant outcomes by probability, matching Argus's Schedule of Prospective Cashflow. Per-lease MLA today; named profiles planned.</t>
+          <t>Argus reports mid-year IRR by default. See irr_summary.annual_mid_year.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>MLA blending</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>OpenVal blends renewal / new-tenant outcomes by probability, matching Argus's Schedule of Prospective Cashflow. Per-lease MLA today; named profiles planned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>Vacancy</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>General vacancy + credit loss are independent deductions on EGI, compounding with MLA downtime. Set general_vacancy_pct=0 to rely solely on MLA-driven absorption vacancy.</t>
         </is>
@@ -1597,10 +1608,10 @@
       <c r="C2" t="n">
         <v>60000</v>
       </c>
-      <c r="D2" s="1" t="n">
+      <c r="D2" s="2" t="n">
         <v>46023</v>
       </c>
-      <c r="E2" s="1" t="n">
+      <c r="E2" s="2" t="n">
         <v>47849</v>
       </c>
       <c r="F2" t="n">
@@ -1641,10 +1652,10 @@
       <c r="C3" t="n">
         <v>40000</v>
       </c>
-      <c r="D3" s="1" t="n">
+      <c r="D3" s="2" t="n">
         <v>46023</v>
       </c>
-      <c r="E3" s="1" t="n">
+      <c r="E3" s="2" t="n">
         <v>47119</v>
       </c>
       <c r="F3" t="n">
@@ -6238,91 +6249,361 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>field</t>
+          <t>line_item</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>Year 1</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Year 3</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Year 5</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>basis</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>forward</t>
-        </is>
-      </c>
+          <t>Rental Revenue</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>terminal_noi</t>
+          <t xml:space="preserve">  Potential Base Rent</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2591899</v>
+        <v>3120000</v>
+      </c>
+      <c r="C3" t="n">
+        <v>3213600</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3310008</v>
+      </c>
+      <c r="E3" t="n">
+        <v>3496730</v>
+      </c>
+      <c r="F3" t="n">
+        <v>3601630</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>gross_sale_price</t>
+          <t xml:space="preserve">  Absorption &amp; Turnover Vacancy</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>37027123</v>
+        <v>0</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-379435</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-35938</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>sale_costs</t>
+          <t xml:space="preserve">  Free Rent</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>740542</v>
+        <v>-300000</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-291951</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>net_sale</t>
+          <t xml:space="preserve">  Scheduled Base Rent</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>36286580</v>
+        <v>2820000</v>
+      </c>
+      <c r="C6" t="n">
+        <v>3213600</v>
+      </c>
+      <c r="D6" t="n">
+        <v>3310008</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2825344</v>
+      </c>
+      <c r="F6" t="n">
+        <v>3565692</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>loan_payoff</t>
+          <t>Total Rental Revenue</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>27075842</v>
+        <v>2820000</v>
+      </c>
+      <c r="C7" t="n">
+        <v>3213600</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3310008</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2825344</v>
+      </c>
+      <c r="F7" t="n">
+        <v>3565692</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>net_sale_to_equity</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>9210738</v>
+          <t>Other Tenant Revenue</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Total Expense Recoveries</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1380000</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1421400</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1464042</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1432565</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1553202</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Total Other Tenant Revenue</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1380000</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1421400</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1464042</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1432565</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1553202</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Total Tenant Revenue</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>4200000</v>
+      </c>
+      <c r="C11" t="n">
+        <v>4635000</v>
+      </c>
+      <c r="D11" t="n">
+        <v>4774050</v>
+      </c>
+      <c r="E11" t="n">
+        <v>4257909</v>
+      </c>
+      <c r="F11" t="n">
+        <v>5118894</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Potential Gross Revenue</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>4200000</v>
+      </c>
+      <c r="C12" t="n">
+        <v>4635000</v>
+      </c>
+      <c r="D12" t="n">
+        <v>4774050</v>
+      </c>
+      <c r="E12" t="n">
+        <v>4257909</v>
+      </c>
+      <c r="F12" t="n">
+        <v>5118894</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Vacancy &amp; Credit Loss</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Vacancy Allowance</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>-156000</v>
+      </c>
+      <c r="C14" t="n">
+        <v>-160680</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-165500</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-155865</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-178285</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Credit Loss</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>-15600</v>
+      </c>
+      <c r="C15" t="n">
+        <v>-16068</v>
+      </c>
+      <c r="D15" t="n">
+        <v>-16550</v>
+      </c>
+      <c r="E15" t="n">
+        <v>-15586</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-17828</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Total Vacancy &amp; Credit Loss</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>-171600</v>
+      </c>
+      <c r="C16" t="n">
+        <v>-176748</v>
+      </c>
+      <c r="D16" t="n">
+        <v>-182050</v>
+      </c>
+      <c r="E16" t="n">
+        <v>-171451</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-196113</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Effective Gross Revenue</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>4028400</v>
+      </c>
+      <c r="C17" t="n">
+        <v>4458252</v>
+      </c>
+      <c r="D17" t="n">
+        <v>4592000</v>
+      </c>
+      <c r="E17" t="n">
+        <v>4086458</v>
+      </c>
+      <c r="F17" t="n">
+        <v>4922781</v>
       </c>
     </row>
   </sheetData>
@@ -6336,112 +6617,92 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>metric</t>
+          <t>field</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>unlevered</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>levered</t>
+          <t>value</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>IRR (monthly_annualized)</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>0.0396</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0.0154</v>
+          <t>basis</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>forward</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>IRR (annual_end_of_year)</t>
+          <t>terminal_noi</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.0387</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0.0144</v>
+        <v>2591899</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>IRR (annual_mid_year)</t>
+          <t>gross_sale_price</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.0436</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.0162</v>
+        <v>37027123</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Equity multiple</t>
+          <t>sale_costs</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1.1875</v>
-      </c>
-      <c r="C5" t="n">
-        <v>1.065</v>
+        <v>740542</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Initial equity</t>
+          <t>net_sale</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>40800000</v>
-      </c>
-      <c r="C6" t="n">
-        <v>16800000</v>
+        <v>36286580</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Going-in cap rate</t>
+          <t>loan_payoff</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.06320000000000001</v>
-      </c>
-      <c r="C7" t="inlineStr"/>
+        <v>27075842</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Stabilized cap rate</t>
+          <t>net_sale_to_equity</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.0728</v>
-      </c>
-      <c r="C8" t="inlineStr"/>
+        <v>9210738</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6454,80 +6715,112 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>year</t>
+          <t>metric</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>noi</t>
+          <t>unlevered</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>yield_on_cost</t>
+          <t>levered</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>2026</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>IRR (monthly_annualized)</t>
+        </is>
       </c>
       <c r="B2" t="n">
-        <v>2528400</v>
+        <v>0.0396</v>
       </c>
       <c r="C2" t="n">
+        <v>0.0154</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>IRR (annual_end_of_year)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.0387</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.0144</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>IRR (annual_mid_year)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.0436</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.0162</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Equity multiple</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1.1875</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1.065</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Initial equity</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>40800000</v>
+      </c>
+      <c r="C6" t="n">
+        <v>16800000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Going-in cap rate</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
         <v>0.06320000000000001</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2027</v>
-      </c>
-      <c r="B3" t="n">
-        <v>2913252</v>
-      </c>
-      <c r="C3" t="n">
+      <c r="C7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Stabilized cap rate</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
         <v>0.0728</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>2028</v>
-      </c>
-      <c r="B4" t="n">
-        <v>3000650</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.075</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>2029</v>
-      </c>
-      <c r="B5" t="n">
-        <v>2447368</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0.0612</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>2030</v>
-      </c>
-      <c r="B6" t="n">
-        <v>3234518</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0.0809</v>
-      </c>
+      <c r="C8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6540,144 +6833,79 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>price $36,000,000</t>
+          <t>noi</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>price $38,000,000</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>price $40,000,000</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>price $42,000,000</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>price $44,000,000</t>
+          <t>yield_on_cost</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>cap 6.000%</t>
-        </is>
+      <c r="A2" t="n">
+        <v>2026</v>
       </c>
       <c r="B2" t="n">
-        <v>0.1025</v>
+        <v>2528400</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0877</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.07389999999999999</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0.061</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0.0488</v>
+        <v>0.06320000000000001</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>cap 6.500%</t>
-        </is>
+      <c r="A3" t="n">
+        <v>2027</v>
       </c>
       <c r="B3" t="n">
-        <v>0.0863</v>
+        <v>2913252</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0716</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.058</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0.0452</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0.0332</v>
+        <v>0.0728</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>cap 7.000%</t>
-        </is>
+      <c r="A4" t="n">
+        <v>2028</v>
       </c>
       <c r="B4" t="n">
-        <v>0.0716</v>
+        <v>3000650</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0571</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.0436</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0.031</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0.0191</v>
+        <v>0.075</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>cap 7.500%</t>
-        </is>
+      <c r="A5" t="n">
+        <v>2029</v>
       </c>
       <c r="B5" t="n">
-        <v>0.0583</v>
+        <v>2447368</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0439</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0.0306</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0.0181</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0.0063</v>
+        <v>0.0612</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>cap 8.000%</t>
-        </is>
+      <c r="A6" t="n">
+        <v>2030</v>
       </c>
       <c r="B6" t="n">
-        <v>0.046</v>
+        <v>3234518</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0318</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0.0186</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0.0062</v>
-      </c>
-      <c r="F6" t="n">
-        <v>-0.0054</v>
+        <v>0.0809</v>
       </c>
     </row>
   </sheetData>
@@ -6691,1169 +6919,144 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">
         <is>
-          <t>lp_distribution</t>
+          <t>price $36,000,000</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>gp_distribution</t>
+          <t>price $38,000,000</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>lp_capital_balance</t>
+          <t>price $40,000,000</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>lp_pref_balance</t>
+          <t>price $42,000,000</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price $44,000,000</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>cap 6.000%</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-954512.42</v>
+        <v>0.1025</v>
       </c>
       <c r="C2" t="n">
-        <v>-106056.94</v>
+        <v>0.0877</v>
       </c>
       <c r="D2" t="n">
-        <v>16074512.42</v>
+        <v>0.07389999999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>100800</v>
+        <v>0.061</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.0488</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>cap 6.500%</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-512.42</v>
+        <v>0.0863</v>
       </c>
       <c r="C3" t="n">
-        <v>-56.94</v>
+        <v>0.0716</v>
       </c>
       <c r="D3" t="n">
-        <v>16075024.85</v>
+        <v>0.058</v>
       </c>
       <c r="E3" t="n">
-        <v>207963.42</v>
+        <v>0.0452</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.0332</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>cap 7.000%</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-512.42</v>
+        <v>0.0716</v>
       </c>
       <c r="C4" t="n">
-        <v>-56.94</v>
+        <v>0.0571</v>
       </c>
       <c r="D4" t="n">
-        <v>16075537.27</v>
+        <v>0.0436</v>
       </c>
       <c r="E4" t="n">
-        <v>315130.25</v>
+        <v>0.031</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.0191</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>cap 7.500%</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>99430.64</v>
+        <v>0.0583</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>0.0439</v>
       </c>
       <c r="D5" t="n">
-        <v>15976106.63</v>
+        <v>0.0306</v>
       </c>
       <c r="E5" t="n">
-        <v>422300.5</v>
+        <v>0.0181</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.0063</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>cap 8.000%</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>99430.64</v>
+        <v>0.046</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>0.0318</v>
       </c>
       <c r="D6" t="n">
-        <v>15876675.99</v>
+        <v>0.0186</v>
       </c>
       <c r="E6" t="n">
-        <v>528807.87</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>99430.64</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" t="n">
-        <v>15777245.35</v>
-      </c>
-      <c r="E7" t="n">
-        <v>634652.38</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>99430.64</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" t="n">
-        <v>15677814.71</v>
-      </c>
-      <c r="E8" t="n">
-        <v>739834.02</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>99430.64</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" t="n">
-        <v>15578384.07</v>
-      </c>
-      <c r="E9" t="n">
-        <v>844352.78</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>99430.64</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" t="n">
-        <v>15478953.43</v>
-      </c>
-      <c r="E10" t="n">
-        <v>948208.6800000001</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>99430.64</v>
-      </c>
-      <c r="C11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" t="n">
-        <v>15379522.8</v>
-      </c>
-      <c r="E11" t="n">
-        <v>1051401.7</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>99430.64</v>
-      </c>
-      <c r="C12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" t="n">
-        <v>15280092.16</v>
-      </c>
-      <c r="E12" t="n">
-        <v>1153931.85</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>99430.64</v>
-      </c>
-      <c r="C13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" t="n">
-        <v>15180661.52</v>
-      </c>
-      <c r="E13" t="n">
-        <v>1255799.13</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2027-01-01</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>94001.64</v>
-      </c>
-      <c r="C14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" t="n">
-        <v>15086659.88</v>
-      </c>
-      <c r="E14" t="n">
-        <v>1357003.54</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2027-02-01</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>94001.64</v>
-      </c>
-      <c r="C15" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" t="n">
-        <v>14992658.24</v>
-      </c>
-      <c r="E15" t="n">
-        <v>1457581.27</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2027-03-01</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>94001.64</v>
-      </c>
-      <c r="C16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" t="n">
-        <v>14898656.6</v>
-      </c>
-      <c r="E16" t="n">
-        <v>1557532.33</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2027-04-01</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>94001.64</v>
-      </c>
-      <c r="C17" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" t="n">
-        <v>14804654.96</v>
-      </c>
-      <c r="E17" t="n">
-        <v>1656856.71</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2027-05-01</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>94001.64</v>
-      </c>
-      <c r="C18" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" t="n">
-        <v>14710653.32</v>
-      </c>
-      <c r="E18" t="n">
-        <v>1755554.41</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>2027-06-01</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>94001.64</v>
-      </c>
-      <c r="C19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" t="n">
-        <v>14616651.68</v>
-      </c>
-      <c r="E19" t="n">
-        <v>1853625.43</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>2027-07-01</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>94001.64</v>
-      </c>
-      <c r="C20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" t="n">
-        <v>14522650.04</v>
-      </c>
-      <c r="E20" t="n">
-        <v>1951069.77</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2027-08-01</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>94001.64</v>
-      </c>
-      <c r="C21" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" t="n">
-        <v>14428648.4</v>
-      </c>
-      <c r="E21" t="n">
-        <v>2047887.44</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2027-09-01</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>94001.64</v>
-      </c>
-      <c r="C22" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" t="n">
-        <v>14334646.76</v>
-      </c>
-      <c r="E22" t="n">
-        <v>2144078.43</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2027-10-01</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>94001.64</v>
-      </c>
-      <c r="C23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" t="n">
-        <v>14240645.12</v>
-      </c>
-      <c r="E23" t="n">
-        <v>2239642.74</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>2027-11-01</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>94001.64</v>
-      </c>
-      <c r="C24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" t="n">
-        <v>14146643.48</v>
-      </c>
-      <c r="E24" t="n">
-        <v>2334580.37</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>2027-12-01</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>94001.64</v>
-      </c>
-      <c r="C25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D25" t="n">
-        <v>14052641.84</v>
-      </c>
-      <c r="E25" t="n">
-        <v>2428891.33</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>2028-01-01</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>113784.77</v>
-      </c>
-      <c r="C26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" t="n">
-        <v>13938857.07</v>
-      </c>
-      <c r="E26" t="n">
-        <v>2522575.61</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>2028-02-01</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>113784.77</v>
-      </c>
-      <c r="C27" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" t="n">
-        <v>13825072.3</v>
-      </c>
-      <c r="E27" t="n">
-        <v>2615501.32</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>2028-03-01</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>113784.77</v>
-      </c>
-      <c r="C28" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" t="n">
-        <v>13711287.53</v>
-      </c>
-      <c r="E28" t="n">
-        <v>2707668.47</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>2028-04-01</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>113784.77</v>
-      </c>
-      <c r="C29" t="n">
-        <v>0</v>
-      </c>
-      <c r="D29" t="n">
-        <v>13597502.76</v>
-      </c>
-      <c r="E29" t="n">
-        <v>2799077.06</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>2028-05-01</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>113784.77</v>
-      </c>
-      <c r="C30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D30" t="n">
-        <v>13483717.99</v>
-      </c>
-      <c r="E30" t="n">
-        <v>2889727.07</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>2028-06-01</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>113784.77</v>
-      </c>
-      <c r="C31" t="n">
-        <v>0</v>
-      </c>
-      <c r="D31" t="n">
-        <v>13369933.22</v>
-      </c>
-      <c r="E31" t="n">
-        <v>2979618.53</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>2028-07-01</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>113784.77</v>
-      </c>
-      <c r="C32" t="n">
-        <v>0</v>
-      </c>
-      <c r="D32" t="n">
-        <v>13256148.45</v>
-      </c>
-      <c r="E32" t="n">
-        <v>3068751.42</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>2028-08-01</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>113784.77</v>
-      </c>
-      <c r="C33" t="n">
-        <v>0</v>
-      </c>
-      <c r="D33" t="n">
-        <v>13142363.68</v>
-      </c>
-      <c r="E33" t="n">
-        <v>3157125.74</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>2028-09-01</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>113784.77</v>
-      </c>
-      <c r="C34" t="n">
-        <v>0</v>
-      </c>
-      <c r="D34" t="n">
-        <v>13028578.91</v>
-      </c>
-      <c r="E34" t="n">
-        <v>3244741.5</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>2028-10-01</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>113784.77</v>
-      </c>
-      <c r="C35" t="n">
-        <v>0</v>
-      </c>
-      <c r="D35" t="n">
-        <v>12914794.14</v>
-      </c>
-      <c r="E35" t="n">
-        <v>3331598.69</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>2028-11-01</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>113784.77</v>
-      </c>
-      <c r="C36" t="n">
-        <v>0</v>
-      </c>
-      <c r="D36" t="n">
-        <v>12801009.37</v>
-      </c>
-      <c r="E36" t="n">
-        <v>3417697.32</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>2028-12-01</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>113784.77</v>
-      </c>
-      <c r="C37" t="n">
-        <v>0</v>
-      </c>
-      <c r="D37" t="n">
-        <v>12687224.6</v>
-      </c>
-      <c r="E37" t="n">
-        <v>3503037.38</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>2029-01-01</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>4687054.07</v>
-      </c>
-      <c r="C38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" t="n">
-        <v>8000170.53</v>
-      </c>
-      <c r="E38" t="n">
-        <v>3587618.88</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>2029-02-01</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>28526.76</v>
-      </c>
-      <c r="C39" t="n">
-        <v>0</v>
-      </c>
-      <c r="D39" t="n">
-        <v>7971643.76</v>
-      </c>
-      <c r="E39" t="n">
-        <v>3640953.35</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>2029-03-01</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>28526.76</v>
-      </c>
-      <c r="C40" t="n">
-        <v>0</v>
-      </c>
-      <c r="D40" t="n">
-        <v>7943117</v>
-      </c>
-      <c r="E40" t="n">
-        <v>3694097.64</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>2029-04-01</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>28526.76</v>
-      </c>
-      <c r="C41" t="n">
-        <v>0</v>
-      </c>
-      <c r="D41" t="n">
-        <v>7914590.23</v>
-      </c>
-      <c r="E41" t="n">
-        <v>3747051.75</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>2029-05-01</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>28526.76</v>
-      </c>
-      <c r="C42" t="n">
-        <v>0</v>
-      </c>
-      <c r="D42" t="n">
-        <v>7886063.47</v>
-      </c>
-      <c r="E42" t="n">
-        <v>3799815.69</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>2029-06-01</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>28526.76</v>
-      </c>
-      <c r="C43" t="n">
-        <v>0</v>
-      </c>
-      <c r="D43" t="n">
-        <v>7857536.71</v>
-      </c>
-      <c r="E43" t="n">
-        <v>3852389.44</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>2029-07-01</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>-345316.69</v>
-      </c>
-      <c r="C44" t="n">
-        <v>-38368.52</v>
-      </c>
-      <c r="D44" t="n">
-        <v>8202853.39</v>
-      </c>
-      <c r="E44" t="n">
-        <v>3904773.02</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>2029-08-01</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>51802.69</v>
-      </c>
-      <c r="C45" t="n">
-        <v>0</v>
-      </c>
-      <c r="D45" t="n">
-        <v>8151050.7</v>
-      </c>
-      <c r="E45" t="n">
-        <v>3959458.71</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>2029-09-01</t>
-        </is>
-      </c>
-      <c r="B46" t="n">
-        <v>51802.69</v>
-      </c>
-      <c r="C46" t="n">
-        <v>0</v>
-      </c>
-      <c r="D46" t="n">
-        <v>8099248.01</v>
-      </c>
-      <c r="E46" t="n">
-        <v>4013799.05</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>2029-10-01</t>
-        </is>
-      </c>
-      <c r="B47" t="n">
-        <v>51802.69</v>
-      </c>
-      <c r="C47" t="n">
-        <v>0</v>
-      </c>
-      <c r="D47" t="n">
-        <v>8047445.32</v>
-      </c>
-      <c r="E47" t="n">
-        <v>4067794.04</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>2029-11-01</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>110949.19</v>
-      </c>
-      <c r="C48" t="n">
-        <v>0</v>
-      </c>
-      <c r="D48" t="n">
-        <v>7936496.13</v>
-      </c>
-      <c r="E48" t="n">
-        <v>4121443.67</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>2029-12-01</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>110949.19</v>
-      </c>
-      <c r="C49" t="n">
-        <v>0</v>
-      </c>
-      <c r="D49" t="n">
-        <v>7825546.94</v>
-      </c>
-      <c r="E49" t="n">
-        <v>4174353.65</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>2030-01-01</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>126832.9</v>
-      </c>
-      <c r="C50" t="n">
-        <v>0</v>
-      </c>
-      <c r="D50" t="n">
-        <v>7698714.04</v>
-      </c>
-      <c r="E50" t="n">
-        <v>4226523.96</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>2030-02-01</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>126832.9</v>
-      </c>
-      <c r="C51" t="n">
-        <v>0</v>
-      </c>
-      <c r="D51" t="n">
-        <v>7571881.15</v>
-      </c>
-      <c r="E51" t="n">
-        <v>4277848.72</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>2030-03-01</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>126832.9</v>
-      </c>
-      <c r="C52" t="n">
-        <v>0</v>
-      </c>
-      <c r="D52" t="n">
-        <v>7445048.25</v>
-      </c>
-      <c r="E52" t="n">
-        <v>4328327.93</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>2030-04-01</t>
-        </is>
-      </c>
-      <c r="B53" t="n">
-        <v>126832.9</v>
-      </c>
-      <c r="C53" t="n">
-        <v>0</v>
-      </c>
-      <c r="D53" t="n">
-        <v>7318215.35</v>
-      </c>
-      <c r="E53" t="n">
-        <v>4377961.58</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>2030-05-01</t>
-        </is>
-      </c>
-      <c r="B54" t="n">
-        <v>126832.9</v>
-      </c>
-      <c r="C54" t="n">
-        <v>0</v>
-      </c>
-      <c r="D54" t="n">
-        <v>7191382.45</v>
-      </c>
-      <c r="E54" t="n">
-        <v>4426749.68</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>2030-06-01</t>
-        </is>
-      </c>
-      <c r="B55" t="n">
-        <v>126832.9</v>
-      </c>
-      <c r="C55" t="n">
-        <v>0</v>
-      </c>
-      <c r="D55" t="n">
-        <v>7064549.56</v>
-      </c>
-      <c r="E55" t="n">
-        <v>4474692.23</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>2030-07-01</t>
-        </is>
-      </c>
-      <c r="B56" t="n">
-        <v>128509.64</v>
-      </c>
-      <c r="C56" t="n">
-        <v>0</v>
-      </c>
-      <c r="D56" t="n">
-        <v>6936039.91</v>
-      </c>
-      <c r="E56" t="n">
-        <v>4521789.23</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>2030-08-01</t>
-        </is>
-      </c>
-      <c r="B57" t="n">
-        <v>128509.64</v>
-      </c>
-      <c r="C57" t="n">
-        <v>0</v>
-      </c>
-      <c r="D57" t="n">
-        <v>6807530.27</v>
-      </c>
-      <c r="E57" t="n">
-        <v>4568029.5</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>2030-09-01</t>
-        </is>
-      </c>
-      <c r="B58" t="n">
-        <v>128509.64</v>
-      </c>
-      <c r="C58" t="n">
-        <v>0</v>
-      </c>
-      <c r="D58" t="n">
-        <v>6679020.63</v>
-      </c>
-      <c r="E58" t="n">
-        <v>4613413.03</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>2030-10-01</t>
-        </is>
-      </c>
-      <c r="B59" t="n">
-        <v>128509.64</v>
-      </c>
-      <c r="C59" t="n">
-        <v>0</v>
-      </c>
-      <c r="D59" t="n">
-        <v>6550510.99</v>
-      </c>
-      <c r="E59" t="n">
-        <v>4657939.84</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>2030-11-01</t>
-        </is>
-      </c>
-      <c r="B60" t="n">
-        <v>128509.64</v>
-      </c>
-      <c r="C60" t="n">
-        <v>0</v>
-      </c>
-      <c r="D60" t="n">
-        <v>6422001.34</v>
-      </c>
-      <c r="E60" t="n">
-        <v>4701609.91</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>2030-12-01</t>
-        </is>
-      </c>
-      <c r="B61" t="n">
-        <v>9339248.140000001</v>
-      </c>
-      <c r="C61" t="n">
-        <v>0</v>
-      </c>
-      <c r="D61" t="n">
-        <v>0</v>
-      </c>
-      <c r="E61" t="n">
-        <v>1827176.45</v>
+        <v>0.0062</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-0.0054</v>
       </c>
     </row>
   </sheetData>
@@ -7862,6 +7065,1182 @@
 </file>
 
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E61"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>lp_distribution</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>gp_distribution</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>lp_capital_balance</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>lp_pref_balance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>-954512.42</v>
+      </c>
+      <c r="C2" t="n">
+        <v>-106056.94</v>
+      </c>
+      <c r="D2" t="n">
+        <v>16074512.42</v>
+      </c>
+      <c r="E2" t="n">
+        <v>100800</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>-512.42</v>
+      </c>
+      <c r="C3" t="n">
+        <v>-56.94</v>
+      </c>
+      <c r="D3" t="n">
+        <v>16075024.85</v>
+      </c>
+      <c r="E3" t="n">
+        <v>207963.42</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>-512.42</v>
+      </c>
+      <c r="C4" t="n">
+        <v>-56.94</v>
+      </c>
+      <c r="D4" t="n">
+        <v>16075537.27</v>
+      </c>
+      <c r="E4" t="n">
+        <v>315130.25</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>99430.64</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>15976106.63</v>
+      </c>
+      <c r="E5" t="n">
+        <v>422300.5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>99430.64</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>15876675.99</v>
+      </c>
+      <c r="E6" t="n">
+        <v>528807.87</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>99430.64</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>15777245.35</v>
+      </c>
+      <c r="E7" t="n">
+        <v>634652.38</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>99430.64</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>15677814.71</v>
+      </c>
+      <c r="E8" t="n">
+        <v>739834.02</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>99430.64</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>15578384.07</v>
+      </c>
+      <c r="E9" t="n">
+        <v>844352.78</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>99430.64</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>15478953.43</v>
+      </c>
+      <c r="E10" t="n">
+        <v>948208.6800000001</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>99430.64</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>15379522.8</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1051401.7</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>99430.64</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" t="n">
+        <v>15280092.16</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1153931.85</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>99430.64</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" t="n">
+        <v>15180661.52</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1255799.13</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2027-01-01</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>94001.64</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" t="n">
+        <v>15086659.88</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1357003.54</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2027-02-01</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>94001.64</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>14992658.24</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1457581.27</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2027-03-01</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>94001.64</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" t="n">
+        <v>14898656.6</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1557532.33</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2027-04-01</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>94001.64</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>14804654.96</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1656856.71</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2027-05-01</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>94001.64</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" t="n">
+        <v>14710653.32</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1755554.41</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2027-06-01</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>94001.64</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" t="n">
+        <v>14616651.68</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1853625.43</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2027-07-01</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>94001.64</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" t="n">
+        <v>14522650.04</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1951069.77</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2027-08-01</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>94001.64</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" t="n">
+        <v>14428648.4</v>
+      </c>
+      <c r="E21" t="n">
+        <v>2047887.44</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2027-09-01</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>94001.64</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" t="n">
+        <v>14334646.76</v>
+      </c>
+      <c r="E22" t="n">
+        <v>2144078.43</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2027-10-01</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>94001.64</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" t="n">
+        <v>14240645.12</v>
+      </c>
+      <c r="E23" t="n">
+        <v>2239642.74</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2027-11-01</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>94001.64</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" t="n">
+        <v>14146643.48</v>
+      </c>
+      <c r="E24" t="n">
+        <v>2334580.37</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2027-12-01</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>94001.64</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" t="n">
+        <v>14052641.84</v>
+      </c>
+      <c r="E25" t="n">
+        <v>2428891.33</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2028-01-01</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>113784.77</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" t="n">
+        <v>13938857.07</v>
+      </c>
+      <c r="E26" t="n">
+        <v>2522575.61</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2028-02-01</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>113784.77</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" t="n">
+        <v>13825072.3</v>
+      </c>
+      <c r="E27" t="n">
+        <v>2615501.32</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2028-03-01</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>113784.77</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" t="n">
+        <v>13711287.53</v>
+      </c>
+      <c r="E28" t="n">
+        <v>2707668.47</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2028-04-01</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>113784.77</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" t="n">
+        <v>13597502.76</v>
+      </c>
+      <c r="E29" t="n">
+        <v>2799077.06</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2028-05-01</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>113784.77</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" t="n">
+        <v>13483717.99</v>
+      </c>
+      <c r="E30" t="n">
+        <v>2889727.07</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2028-06-01</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>113784.77</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" t="n">
+        <v>13369933.22</v>
+      </c>
+      <c r="E31" t="n">
+        <v>2979618.53</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2028-07-01</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>113784.77</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" t="n">
+        <v>13256148.45</v>
+      </c>
+      <c r="E32" t="n">
+        <v>3068751.42</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2028-08-01</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>113784.77</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" t="n">
+        <v>13142363.68</v>
+      </c>
+      <c r="E33" t="n">
+        <v>3157125.74</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2028-09-01</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>113784.77</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" t="n">
+        <v>13028578.91</v>
+      </c>
+      <c r="E34" t="n">
+        <v>3244741.5</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2028-10-01</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>113784.77</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" t="n">
+        <v>12914794.14</v>
+      </c>
+      <c r="E35" t="n">
+        <v>3331598.69</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2028-11-01</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>113784.77</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" t="n">
+        <v>12801009.37</v>
+      </c>
+      <c r="E36" t="n">
+        <v>3417697.32</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2028-12-01</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>113784.77</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" t="n">
+        <v>12687224.6</v>
+      </c>
+      <c r="E37" t="n">
+        <v>3503037.38</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2029-01-01</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>4687054.07</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" t="n">
+        <v>8000170.53</v>
+      </c>
+      <c r="E38" t="n">
+        <v>3587618.88</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2029-02-01</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>28526.76</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" t="n">
+        <v>7971643.76</v>
+      </c>
+      <c r="E39" t="n">
+        <v>3640953.35</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2029-03-01</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>28526.76</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" t="n">
+        <v>7943117</v>
+      </c>
+      <c r="E40" t="n">
+        <v>3694097.64</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2029-04-01</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>28526.76</v>
+      </c>
+      <c r="C41" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" t="n">
+        <v>7914590.23</v>
+      </c>
+      <c r="E41" t="n">
+        <v>3747051.75</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2029-05-01</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>28526.76</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" t="n">
+        <v>7886063.47</v>
+      </c>
+      <c r="E42" t="n">
+        <v>3799815.69</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2029-06-01</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>28526.76</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" t="n">
+        <v>7857536.71</v>
+      </c>
+      <c r="E43" t="n">
+        <v>3852389.44</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2029-07-01</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>-345316.69</v>
+      </c>
+      <c r="C44" t="n">
+        <v>-38368.52</v>
+      </c>
+      <c r="D44" t="n">
+        <v>8202853.39</v>
+      </c>
+      <c r="E44" t="n">
+        <v>3904773.02</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2029-08-01</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>51802.69</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" t="n">
+        <v>8151050.7</v>
+      </c>
+      <c r="E45" t="n">
+        <v>3959458.71</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2029-09-01</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>51802.69</v>
+      </c>
+      <c r="C46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" t="n">
+        <v>8099248.01</v>
+      </c>
+      <c r="E46" t="n">
+        <v>4013799.05</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2029-10-01</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>51802.69</v>
+      </c>
+      <c r="C47" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" t="n">
+        <v>8047445.32</v>
+      </c>
+      <c r="E47" t="n">
+        <v>4067794.04</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2029-11-01</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>110949.19</v>
+      </c>
+      <c r="C48" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" t="n">
+        <v>7936496.13</v>
+      </c>
+      <c r="E48" t="n">
+        <v>4121443.67</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2029-12-01</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>110949.19</v>
+      </c>
+      <c r="C49" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" t="n">
+        <v>7825546.94</v>
+      </c>
+      <c r="E49" t="n">
+        <v>4174353.65</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2030-01-01</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>126832.9</v>
+      </c>
+      <c r="C50" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" t="n">
+        <v>7698714.04</v>
+      </c>
+      <c r="E50" t="n">
+        <v>4226523.96</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2030-02-01</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>126832.9</v>
+      </c>
+      <c r="C51" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" t="n">
+        <v>7571881.15</v>
+      </c>
+      <c r="E51" t="n">
+        <v>4277848.72</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2030-03-01</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>126832.9</v>
+      </c>
+      <c r="C52" t="n">
+        <v>0</v>
+      </c>
+      <c r="D52" t="n">
+        <v>7445048.25</v>
+      </c>
+      <c r="E52" t="n">
+        <v>4328327.93</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2030-04-01</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>126832.9</v>
+      </c>
+      <c r="C53" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" t="n">
+        <v>7318215.35</v>
+      </c>
+      <c r="E53" t="n">
+        <v>4377961.58</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2030-05-01</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>126832.9</v>
+      </c>
+      <c r="C54" t="n">
+        <v>0</v>
+      </c>
+      <c r="D54" t="n">
+        <v>7191382.45</v>
+      </c>
+      <c r="E54" t="n">
+        <v>4426749.68</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2030-06-01</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>126832.9</v>
+      </c>
+      <c r="C55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D55" t="n">
+        <v>7064549.56</v>
+      </c>
+      <c r="E55" t="n">
+        <v>4474692.23</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2030-07-01</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>128509.64</v>
+      </c>
+      <c r="C56" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" t="n">
+        <v>6936039.91</v>
+      </c>
+      <c r="E56" t="n">
+        <v>4521789.23</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2030-08-01</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>128509.64</v>
+      </c>
+      <c r="C57" t="n">
+        <v>0</v>
+      </c>
+      <c r="D57" t="n">
+        <v>6807530.27</v>
+      </c>
+      <c r="E57" t="n">
+        <v>4568029.5</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2030-09-01</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>128509.64</v>
+      </c>
+      <c r="C58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D58" t="n">
+        <v>6679020.63</v>
+      </c>
+      <c r="E58" t="n">
+        <v>4613413.03</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2030-10-01</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>128509.64</v>
+      </c>
+      <c r="C59" t="n">
+        <v>0</v>
+      </c>
+      <c r="D59" t="n">
+        <v>6550510.99</v>
+      </c>
+      <c r="E59" t="n">
+        <v>4657939.84</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2030-11-01</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>128509.64</v>
+      </c>
+      <c r="C60" t="n">
+        <v>0</v>
+      </c>
+      <c r="D60" t="n">
+        <v>6422001.34</v>
+      </c>
+      <c r="E60" t="n">
+        <v>4701609.91</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2030-12-01</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>9339248.140000001</v>
+      </c>
+      <c r="C61" t="n">
+        <v>0</v>
+      </c>
+      <c r="D61" t="n">
+        <v>0</v>
+      </c>
+      <c r="E61" t="n">
+        <v>1827176.45</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>